<commit_message>
LMDI: Rydd README og sett status til aktiv
- Oppdater Plan-seksjonen fra 1.0.x til 1.x-serien
- Endre presens til fortid for FHIR R4-utvikling
- Sett status fra draft til active i sushi-config.yaml

Lukker #18 f50b8f66a83944c2a6ab6f92af82decef7dbb95b
</commit_message>
<xml_diff>
--- a/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
+++ b/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-08T10:26:49+00:00</t>
+    <t>2026-04-08T10:36:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
LMDI: Merge pull request #111 from folkehelseinstituttet/roar/versjon-1.1.4
Bump til 1.1.4 og rett avvik i README-tabellen 1f597673ed5e2dbb8caf7a16541bfcd40e40f44a
</commit_message>
<xml_diff>
--- a/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
+++ b/currentbuild/CodeSystem-LokalLegemiddelkatalogCodeSystem.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.3</t>
+    <t>1.1.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T06:55:15+00:00</t>
+    <t>2026-08-24T07:23:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>